<commit_message>
📊 Actualizar METAS_MES_PF.xlsx — 08-04-2026, 12:06:09 p. m.
</commit_message>
<xml_diff>
--- a/datos/METAS_MES_PF.xlsx
+++ b/datos/METAS_MES_PF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{53E4F5CA-E421-4DEA-BC20-EED8B6470087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{411EF0C0-189E-40C0-A86A-729F27F74422}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{AC73539F-EBD3-477C-B1DA-3F37369700C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A55034A-A8A1-4A29-AFAE-8DE20E7C0F05}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7E8DF223-1267-404B-9AAA-1657BEB8CA32}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Lider</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Camilo Medel</t>
   </si>
   <si>
-    <t>Humberto Barbiery</t>
-  </si>
-  <si>
     <t>Meta marzo Proteccion Familiar</t>
   </si>
   <si>
@@ -69,6 +66,15 @@
   </si>
   <si>
     <t>Meta Cantidad de Contratos</t>
+  </si>
+  <si>
+    <t>Patricia martinez</t>
+  </si>
+  <si>
+    <t>Sugey Vivas</t>
+  </si>
+  <si>
+    <t>Raul Bustos</t>
   </si>
 </sst>
 </file>
@@ -135,7 +141,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -145,6 +151,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
@@ -480,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00254501-E372-48E8-93B0-FF6CCCB5CFBB}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
@@ -490,7 +500,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -498,17 +508,17 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="7">
         <v>25000000</v>
       </c>
       <c r="C3" s="6">
@@ -524,7 +534,7 @@
         <v>120000000</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" ref="C4:C9" si="0">ROUNDUP(B4/1750000,0)</f>
+        <f t="shared" ref="C4:C10" si="0">ROUNDUP(B4/1750000,0)</f>
         <v>69</v>
       </c>
     </row>
@@ -532,7 +542,7 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="8">
         <v>25000000</v>
       </c>
       <c r="C5" s="6">
@@ -544,7 +554,7 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="8">
         <v>25000000</v>
       </c>
       <c r="C6" s="6">
@@ -556,7 +566,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="8">
         <v>25000000</v>
       </c>
       <c r="C7" s="6">
@@ -566,9 +576,9 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4">
+        <v>10</v>
+      </c>
+      <c r="B8" s="7">
         <v>10000000</v>
       </c>
       <c r="C8" s="6">
@@ -577,16 +587,40 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="5">
-        <f>SUM(B3:B8)</f>
-        <v>230000000</v>
-      </c>
-      <c r="C9" s="5">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="7">
+        <v>10000000</v>
+      </c>
+      <c r="C9" s="6">
         <f t="shared" si="0"/>
-        <v>132</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="7">
+        <v>10000000</v>
+      </c>
+      <c r="C10" s="6">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5">
+        <f>SUM(B3:B10)</f>
+        <v>250000000</v>
+      </c>
+      <c r="C11" s="5">
+        <f>ROUNDUP(B11/1750000,0)</f>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>